<commit_message>
viết tài liệu hướng dẫn chi tiết
</commit_message>
<xml_diff>
--- a/docs/Danh sách thành viên và phân chia công việc.xlsx
+++ b/docs/Danh sách thành viên và phân chia công việc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\tranmanhlinh\Code\Manhlinh's project\ProductManagement\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910CB960-ABC9-4A10-BCDF-5301B31C1D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41C82FA8-61E8-430B-908A-832155E9B1DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="2" xr2:uid="{CA9928F4-C8DF-4BAD-BBAB-130F73E75540}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{CA9928F4-C8DF-4BAD-BBAB-130F73E75540}"/>
   </bookViews>
   <sheets>
     <sheet name="Thành viên nhóm" sheetId="3" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="76">
   <si>
     <t>Hệ thống quản lý sản phẩm bằng mã vạch</t>
   </si>
@@ -261,6 +261,9 @@
   </si>
   <si>
     <t xml:space="preserve">Hoàn thiện video, slide, báo cáo </t>
+  </si>
+  <si>
+    <t>Mạnh Linh, Thái Hưng</t>
   </si>
 </sst>
 </file>
@@ -298,12 +301,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="8">
@@ -406,7 +415,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -427,6 +436,15 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -454,6 +472,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -478,18 +499,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -833,42 +852,42 @@
       <c r="H4" s="7"/>
     </row>
     <row r="5" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="25"/>
-      <c r="F5" s="26" t="s">
+      <c r="E5" s="9"/>
+      <c r="F5" s="10" t="s">
         <v>32</v>
       </c>
-      <c r="G5" s="26"/>
-      <c r="H5" s="26"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
     </row>
     <row r="6" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="25"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="25"/>
-      <c r="H6" s="25"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
     </row>
     <row r="7" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="25"/>
-      <c r="F7" s="25"/>
-      <c r="G7" s="25"/>
-      <c r="H7" s="25"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
     </row>
     <row r="8" spans="4:8" x14ac:dyDescent="0.3">
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="25"/>
-      <c r="F8" s="25"/>
-      <c r="G8" s="25"/>
-      <c r="H8" s="25"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -918,72 +937,72 @@
       <c r="C5" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="E5" s="25"/>
+      <c r="E5" s="9"/>
     </row>
     <row r="6" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C6" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="25" t="s">
+      <c r="D6" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="E6" s="25"/>
+      <c r="E6" s="9"/>
     </row>
     <row r="7" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C7" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D7" s="25" t="s">
+      <c r="D7" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="25"/>
+      <c r="E7" s="9"/>
     </row>
     <row r="8" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="25" t="s">
+      <c r="D8" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="E8" s="25"/>
+      <c r="E8" s="9"/>
     </row>
     <row r="9" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C9" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="25" t="s">
+      <c r="D9" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="E9" s="25"/>
+      <c r="E9" s="9"/>
     </row>
     <row r="10" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C10" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="D10" s="25" t="s">
+      <c r="D10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="E10" s="25"/>
+      <c r="E10" s="9"/>
     </row>
     <row r="11" spans="3:5" x14ac:dyDescent="0.3">
       <c r="C11" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="25" t="s">
+      <c r="D11" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="25"/>
+      <c r="E11" s="9"/>
     </row>
     <row r="12" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="D12" s="27"/>
-      <c r="E12" s="27"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
     </row>
     <row r="13" spans="3:5" x14ac:dyDescent="0.3">
-      <c r="D13" s="27"/>
-      <c r="E13" s="27"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -1042,803 +1061,803 @@
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="8" t="s">
+      <c r="K4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="L4" s="9"/>
-      <c r="M4" s="10"/>
+      <c r="L4" s="12"/>
+      <c r="M4" s="13"/>
     </row>
     <row r="5" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C5" s="1">
         <v>6</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="D5" s="17" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14" t="s">
+      <c r="E5" s="17"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="17"/>
+      <c r="H5" s="17"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="17"/>
+      <c r="K5" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
+      <c r="L5" s="17"/>
+      <c r="M5" s="17"/>
     </row>
     <row r="6" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C6" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="14" t="s">
+      <c r="D6" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-      <c r="G6" s="14"/>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14" t="s">
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+      <c r="H6" s="17"/>
+      <c r="I6" s="17"/>
+      <c r="J6" s="17"/>
+      <c r="K6" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
+      <c r="L6" s="17"/>
+      <c r="M6" s="17"/>
     </row>
     <row r="7" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="D7" s="17" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-      <c r="G7" s="14"/>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14" t="s">
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
+      <c r="G7" s="17"/>
+      <c r="H7" s="17"/>
+      <c r="I7" s="17"/>
+      <c r="J7" s="17"/>
+      <c r="K7" s="17" t="s">
         <v>13</v>
       </c>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
+      <c r="L7" s="17"/>
+      <c r="M7" s="17"/>
     </row>
     <row r="8" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C8" s="1">
         <v>9</v>
       </c>
-      <c r="D8" s="14" t="s">
+      <c r="D8" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14" t="s">
+      <c r="E8" s="17"/>
+      <c r="F8" s="17"/>
+      <c r="G8" s="17"/>
+      <c r="H8" s="17"/>
+      <c r="I8" s="17"/>
+      <c r="J8" s="17"/>
+      <c r="K8" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
+      <c r="L8" s="17"/>
+      <c r="M8" s="17"/>
     </row>
     <row r="12" spans="3:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="17"/>
-      <c r="E12" s="17"/>
-      <c r="F12" s="17"/>
-      <c r="G12" s="17"/>
-      <c r="H12" s="17"/>
-      <c r="I12" s="17"/>
-      <c r="J12" s="17"/>
-      <c r="K12" s="17"/>
-      <c r="L12" s="17"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="17"/>
-      <c r="O12" s="17"/>
-      <c r="P12" s="17"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="21"/>
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+      <c r="L12" s="21"/>
+      <c r="M12" s="21"/>
+      <c r="N12" s="21"/>
+      <c r="O12" s="21"/>
+      <c r="P12" s="21"/>
     </row>
     <row r="13" spans="3:16" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C13" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="E13" s="11"/>
-      <c r="F13" s="11" t="s">
+      <c r="E13" s="14"/>
+      <c r="F13" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="11"/>
-      <c r="H13" s="11"/>
-      <c r="I13" s="11"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="12" t="s">
+      <c r="G13" s="14"/>
+      <c r="H13" s="14"/>
+      <c r="I13" s="14"/>
+      <c r="J13" s="14"/>
+      <c r="K13" s="15" t="s">
         <v>21</v>
       </c>
-      <c r="L13" s="13"/>
-      <c r="M13" s="11" t="s">
+      <c r="L13" s="16"/>
+      <c r="M13" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="N13" s="11"/>
-      <c r="O13" s="17" t="s">
+      <c r="N13" s="14"/>
+      <c r="O13" s="21" t="s">
         <v>50</v>
       </c>
-      <c r="P13" s="15"/>
+      <c r="P13" s="18"/>
     </row>
     <row r="14" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C14" s="5">
         <v>6</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15" t="s">
+      <c r="E14" s="18"/>
+      <c r="F14" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="15"/>
-      <c r="K14" s="15" t="s">
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="18"/>
+      <c r="J14" s="18"/>
+      <c r="K14" s="18" t="s">
         <v>13</v>
       </c>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15" t="s">
+      <c r="L14" s="18"/>
+      <c r="M14" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="N14" s="15"/>
-      <c r="O14" s="16"/>
-      <c r="P14" s="16"/>
+      <c r="N14" s="18"/>
+      <c r="O14" s="19"/>
+      <c r="P14" s="19"/>
     </row>
     <row r="15" spans="3:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="5">
         <v>7</v>
       </c>
-      <c r="D15" s="15" t="s">
+      <c r="D15" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15" t="s">
+      <c r="E15" s="18"/>
+      <c r="F15" s="18" t="s">
         <v>40</v>
       </c>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15"/>
-      <c r="K15" s="15" t="s">
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15" t="s">
+      <c r="L15" s="18"/>
+      <c r="M15" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="N15" s="15"/>
-      <c r="O15" s="16" t="s">
+      <c r="N15" s="18"/>
+      <c r="O15" s="19" t="s">
         <v>48</v>
       </c>
-      <c r="P15" s="16"/>
+      <c r="P15" s="19"/>
     </row>
     <row r="16" spans="3:16" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C16" s="5">
         <v>7</v>
       </c>
-      <c r="D16" s="15" t="s">
+      <c r="D16" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15" t="s">
+      <c r="E16" s="18"/>
+      <c r="F16" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="15"/>
-      <c r="K16" s="15" t="s">
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="18"/>
+      <c r="J16" s="18"/>
+      <c r="K16" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15" t="s">
+      <c r="L16" s="18"/>
+      <c r="M16" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="N16" s="15"/>
-      <c r="O16" s="16" t="s">
+      <c r="N16" s="18"/>
+      <c r="O16" s="19" t="s">
         <v>47</v>
       </c>
-      <c r="P16" s="16"/>
+      <c r="P16" s="19"/>
     </row>
     <row r="17" spans="3:16" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C17" s="5">
         <v>7</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15" t="s">
+      <c r="E17" s="18"/>
+      <c r="F17" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="G17" s="15"/>
-      <c r="H17" s="15"/>
-      <c r="I17" s="15"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="15" t="s">
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="L17" s="15"/>
-      <c r="M17" s="15" t="s">
+      <c r="L17" s="18"/>
+      <c r="M17" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="N17" s="15"/>
-      <c r="O17" s="16" t="s">
+      <c r="N17" s="18"/>
+      <c r="O17" s="19" t="s">
         <v>51</v>
       </c>
-      <c r="P17" s="16"/>
+      <c r="P17" s="19"/>
     </row>
     <row r="18" spans="3:16" ht="46.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C18" s="5">
         <v>7</v>
       </c>
-      <c r="D18" s="15" t="s">
+      <c r="D18" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15" t="s">
+      <c r="E18" s="18"/>
+      <c r="F18" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="G18" s="15"/>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="16" t="s">
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="18"/>
+      <c r="J18" s="18"/>
+      <c r="K18" s="19" t="s">
         <v>39</v>
       </c>
-      <c r="L18" s="16"/>
-      <c r="M18" s="15" t="s">
+      <c r="L18" s="19"/>
+      <c r="M18" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="N18" s="15"/>
-      <c r="O18" s="16"/>
-      <c r="P18" s="16"/>
+      <c r="N18" s="18"/>
+      <c r="O18" s="19"/>
+      <c r="P18" s="19"/>
     </row>
     <row r="19" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C19" s="5">
         <v>8</v>
       </c>
-      <c r="D19" s="15" t="s">
+      <c r="D19" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="E19" s="15"/>
-      <c r="F19" s="18" t="s">
+      <c r="E19" s="18"/>
+      <c r="F19" s="22" t="s">
         <v>61</v>
       </c>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="19"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="21" t="s">
+      <c r="G19" s="23"/>
+      <c r="H19" s="23"/>
+      <c r="I19" s="23"/>
+      <c r="J19" s="24"/>
+      <c r="K19" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="L19" s="22"/>
-      <c r="M19" s="18" t="s">
+      <c r="L19" s="26"/>
+      <c r="M19" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="N19" s="20"/>
-      <c r="O19" s="23"/>
-      <c r="P19" s="24"/>
+      <c r="N19" s="24"/>
+      <c r="O19" s="27"/>
+      <c r="P19" s="28"/>
     </row>
     <row r="20" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C20" s="5">
         <v>8</v>
       </c>
-      <c r="D20" s="15" t="s">
+      <c r="D20" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="E20" s="15"/>
-      <c r="F20" s="15" t="s">
+      <c r="E20" s="18"/>
+      <c r="F20" s="18" t="s">
         <v>64</v>
       </c>
-      <c r="G20" s="15"/>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15" t="s">
-        <v>65</v>
-      </c>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15" t="s">
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="18"/>
+      <c r="J20" s="18"/>
+      <c r="K20" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="L20" s="18"/>
+      <c r="M20" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="N20" s="15"/>
-      <c r="O20" s="16"/>
-      <c r="P20" s="16"/>
-    </row>
-    <row r="21" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="5">
+      <c r="N20" s="18"/>
+      <c r="O20" s="19"/>
+      <c r="P20" s="19"/>
+    </row>
+    <row r="21" spans="3:16" s="32" customFormat="1" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C21" s="29">
         <v>8</v>
       </c>
-      <c r="D21" s="15" t="s">
+      <c r="D21" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="E21" s="15"/>
-      <c r="F21" s="15" t="s">
+      <c r="E21" s="30"/>
+      <c r="F21" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15" t="s">
+      <c r="G21" s="30"/>
+      <c r="H21" s="30"/>
+      <c r="I21" s="30"/>
+      <c r="J21" s="30"/>
+      <c r="K21" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="L21" s="15"/>
-      <c r="M21" s="15" t="s">
+      <c r="L21" s="30"/>
+      <c r="M21" s="30" t="s">
         <v>68</v>
       </c>
-      <c r="N21" s="15"/>
-      <c r="O21" s="16"/>
-      <c r="P21" s="16"/>
+      <c r="N21" s="30"/>
+      <c r="O21" s="31"/>
+      <c r="P21" s="31"/>
     </row>
     <row r="22" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C22" s="5">
         <v>8</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D22" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="E22" s="15"/>
-      <c r="F22" s="15" t="s">
+      <c r="E22" s="18"/>
+      <c r="F22" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15" t="s">
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="18"/>
+      <c r="J22" s="18"/>
+      <c r="K22" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15" t="s">
+      <c r="L22" s="18"/>
+      <c r="M22" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="N22" s="15"/>
-      <c r="O22" s="16"/>
-      <c r="P22" s="16"/>
+      <c r="N22" s="18"/>
+      <c r="O22" s="19"/>
+      <c r="P22" s="19"/>
     </row>
     <row r="23" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C23" s="5">
         <v>8</v>
       </c>
-      <c r="D23" s="15" t="s">
+      <c r="D23" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15" t="s">
+      <c r="E23" s="18"/>
+      <c r="F23" s="18" t="s">
         <v>72</v>
       </c>
-      <c r="G23" s="15"/>
-      <c r="H23" s="15"/>
-      <c r="I23" s="15"/>
-      <c r="J23" s="15"/>
-      <c r="K23" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="L23" s="15"/>
-      <c r="M23" s="28">
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="18"/>
+      <c r="J23" s="18"/>
+      <c r="K23" s="18" t="s">
+        <v>65</v>
+      </c>
+      <c r="L23" s="18"/>
+      <c r="M23" s="20">
         <v>46033</v>
       </c>
-      <c r="N23" s="15"/>
-      <c r="O23" s="16"/>
-      <c r="P23" s="16"/>
+      <c r="N23" s="18"/>
+      <c r="O23" s="19"/>
+      <c r="P23" s="19"/>
     </row>
     <row r="24" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C24" s="5">
         <v>8</v>
       </c>
-      <c r="D24" s="15" t="s">
+      <c r="D24" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15" t="s">
+      <c r="E24" s="18"/>
+      <c r="F24" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15" t="s">
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="18"/>
+      <c r="J24" s="18"/>
+      <c r="K24" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="L24" s="15"/>
-      <c r="M24" s="28">
+      <c r="L24" s="18"/>
+      <c r="M24" s="20">
         <v>46064</v>
       </c>
-      <c r="N24" s="15"/>
-      <c r="O24" s="16"/>
-      <c r="P24" s="16"/>
+      <c r="N24" s="18"/>
+      <c r="O24" s="19"/>
+      <c r="P24" s="19"/>
     </row>
     <row r="25" spans="3:16" ht="21" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C25" s="5">
         <v>9</v>
       </c>
-      <c r="D25" s="28">
+      <c r="D25" s="20">
         <v>46033</v>
       </c>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15" t="s">
+      <c r="E25" s="18"/>
+      <c r="F25" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="G25" s="15"/>
-      <c r="H25" s="15"/>
-      <c r="I25" s="15"/>
-      <c r="J25" s="15"/>
-      <c r="K25" s="15" t="s">
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="18"/>
+      <c r="J25" s="18"/>
+      <c r="K25" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="L25" s="15"/>
-      <c r="M25" s="28">
+      <c r="L25" s="18"/>
+      <c r="M25" s="20">
         <v>46092</v>
       </c>
-      <c r="N25" s="15"/>
-      <c r="O25" s="16"/>
-      <c r="P25" s="16"/>
+      <c r="N25" s="18"/>
+      <c r="O25" s="19"/>
+      <c r="P25" s="19"/>
     </row>
     <row r="26" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C26" s="5"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="15"/>
-      <c r="K26" s="15"/>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="15"/>
-      <c r="O26" s="16"/>
-      <c r="P26" s="16"/>
+      <c r="D26" s="18"/>
+      <c r="E26" s="18"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="18"/>
+      <c r="J26" s="18"/>
+      <c r="K26" s="18"/>
+      <c r="L26" s="18"/>
+      <c r="M26" s="18"/>
+      <c r="N26" s="18"/>
+      <c r="O26" s="19"/>
+      <c r="P26" s="19"/>
     </row>
     <row r="27" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C27" s="5"/>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15"/>
-      <c r="K27" s="15"/>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
-      <c r="N27" s="15"/>
-      <c r="O27" s="16"/>
-      <c r="P27" s="16"/>
+      <c r="D27" s="18"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="18"/>
+      <c r="J27" s="18"/>
+      <c r="K27" s="18"/>
+      <c r="L27" s="18"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="18"/>
+      <c r="O27" s="19"/>
+      <c r="P27" s="19"/>
     </row>
     <row r="28" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C28" s="5"/>
-      <c r="D28" s="15"/>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
-      <c r="G28" s="15"/>
-      <c r="H28" s="15"/>
-      <c r="I28" s="15"/>
-      <c r="J28" s="15"/>
-      <c r="K28" s="15"/>
-      <c r="L28" s="15"/>
-      <c r="M28" s="15"/>
-      <c r="N28" s="15"/>
-      <c r="O28" s="16"/>
-      <c r="P28" s="16"/>
+      <c r="D28" s="18"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="18"/>
+      <c r="J28" s="18"/>
+      <c r="K28" s="18"/>
+      <c r="L28" s="18"/>
+      <c r="M28" s="18"/>
+      <c r="N28" s="18"/>
+      <c r="O28" s="19"/>
+      <c r="P28" s="19"/>
     </row>
     <row r="29" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C29" s="5"/>
-      <c r="D29" s="15"/>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="15"/>
-      <c r="K29" s="15"/>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="16"/>
-      <c r="P29" s="16"/>
+      <c r="D29" s="18"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="18"/>
+      <c r="J29" s="18"/>
+      <c r="K29" s="18"/>
+      <c r="L29" s="18"/>
+      <c r="M29" s="18"/>
+      <c r="N29" s="18"/>
+      <c r="O29" s="19"/>
+      <c r="P29" s="19"/>
     </row>
     <row r="30" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C30" s="5"/>
-      <c r="D30" s="15"/>
-      <c r="E30" s="15"/>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15"/>
-      <c r="H30" s="15"/>
-      <c r="I30" s="15"/>
-      <c r="J30" s="15"/>
-      <c r="K30" s="15"/>
-      <c r="L30" s="15"/>
-      <c r="M30" s="15"/>
-      <c r="N30" s="15"/>
-      <c r="O30" s="16"/>
-      <c r="P30" s="16"/>
+      <c r="D30" s="18"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="18"/>
+      <c r="J30" s="18"/>
+      <c r="K30" s="18"/>
+      <c r="L30" s="18"/>
+      <c r="M30" s="18"/>
+      <c r="N30" s="18"/>
+      <c r="O30" s="19"/>
+      <c r="P30" s="19"/>
     </row>
     <row r="31" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C31" s="5"/>
-      <c r="D31" s="15"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15"/>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="16"/>
-      <c r="P31" s="16"/>
+      <c r="D31" s="18"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="18"/>
+      <c r="J31" s="18"/>
+      <c r="K31" s="18"/>
+      <c r="L31" s="18"/>
+      <c r="M31" s="18"/>
+      <c r="N31" s="18"/>
+      <c r="O31" s="19"/>
+      <c r="P31" s="19"/>
     </row>
     <row r="32" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C32" s="5"/>
-      <c r="D32" s="15"/>
-      <c r="E32" s="15"/>
-      <c r="F32" s="15"/>
-      <c r="G32" s="15"/>
-      <c r="H32" s="15"/>
-      <c r="I32" s="15"/>
-      <c r="J32" s="15"/>
-      <c r="K32" s="15"/>
-      <c r="L32" s="15"/>
-      <c r="M32" s="15"/>
-      <c r="N32" s="15"/>
-      <c r="O32" s="16"/>
-      <c r="P32" s="16"/>
+      <c r="D32" s="18"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+      <c r="N32" s="18"/>
+      <c r="O32" s="19"/>
+      <c r="P32" s="19"/>
     </row>
     <row r="33" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C33" s="5"/>
-      <c r="D33" s="15"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
-      <c r="K33" s="15"/>
-      <c r="L33" s="15"/>
-      <c r="M33" s="15"/>
-      <c r="N33" s="15"/>
-      <c r="O33" s="16"/>
-      <c r="P33" s="16"/>
+      <c r="D33" s="18"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="18"/>
+      <c r="J33" s="18"/>
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+      <c r="N33" s="18"/>
+      <c r="O33" s="19"/>
+      <c r="P33" s="19"/>
     </row>
     <row r="34" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C34" s="5"/>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15"/>
-      <c r="G34" s="15"/>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="N34" s="15"/>
-      <c r="O34" s="16"/>
-      <c r="P34" s="16"/>
+      <c r="D34" s="18"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="18"/>
+      <c r="J34" s="18"/>
+      <c r="K34" s="18"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="18"/>
+      <c r="N34" s="18"/>
+      <c r="O34" s="19"/>
+      <c r="P34" s="19"/>
     </row>
     <row r="35" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C35" s="5"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="16"/>
-      <c r="P35" s="16"/>
+      <c r="D35" s="18"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="18"/>
+      <c r="J35" s="18"/>
+      <c r="K35" s="18"/>
+      <c r="L35" s="18"/>
+      <c r="M35" s="18"/>
+      <c r="N35" s="18"/>
+      <c r="O35" s="19"/>
+      <c r="P35" s="19"/>
     </row>
     <row r="36" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C36" s="5"/>
-      <c r="D36" s="15"/>
-      <c r="E36" s="15"/>
-      <c r="F36" s="15"/>
-      <c r="G36" s="15"/>
-      <c r="H36" s="15"/>
-      <c r="I36" s="15"/>
-      <c r="J36" s="15"/>
-      <c r="K36" s="15"/>
-      <c r="L36" s="15"/>
-      <c r="M36" s="15"/>
-      <c r="N36" s="15"/>
-      <c r="O36" s="16"/>
-      <c r="P36" s="16"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="18"/>
+      <c r="K36" s="18"/>
+      <c r="L36" s="18"/>
+      <c r="M36" s="18"/>
+      <c r="N36" s="18"/>
+      <c r="O36" s="19"/>
+      <c r="P36" s="19"/>
     </row>
     <row r="37" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C37" s="5"/>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
-      <c r="F37" s="15"/>
-      <c r="G37" s="15"/>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
-      <c r="K37" s="15"/>
-      <c r="L37" s="15"/>
-      <c r="M37" s="15"/>
-      <c r="N37" s="15"/>
-      <c r="O37" s="16"/>
-      <c r="P37" s="16"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="18"/>
+      <c r="J37" s="18"/>
+      <c r="K37" s="18"/>
+      <c r="L37" s="18"/>
+      <c r="M37" s="18"/>
+      <c r="N37" s="18"/>
+      <c r="O37" s="19"/>
+      <c r="P37" s="19"/>
     </row>
     <row r="38" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C38" s="5"/>
-      <c r="D38" s="15"/>
-      <c r="E38" s="15"/>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="15"/>
-      <c r="I38" s="15"/>
-      <c r="J38" s="15"/>
-      <c r="K38" s="15"/>
-      <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
-      <c r="N38" s="15"/>
-      <c r="O38" s="16"/>
-      <c r="P38" s="16"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="18"/>
+      <c r="J38" s="18"/>
+      <c r="K38" s="18"/>
+      <c r="L38" s="18"/>
+      <c r="M38" s="18"/>
+      <c r="N38" s="18"/>
+      <c r="O38" s="19"/>
+      <c r="P38" s="19"/>
     </row>
     <row r="39" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C39" s="5"/>
-      <c r="D39" s="15"/>
-      <c r="E39" s="15"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15"/>
-      <c r="H39" s="15"/>
-      <c r="I39" s="15"/>
-      <c r="J39" s="15"/>
-      <c r="K39" s="15"/>
-      <c r="L39" s="15"/>
-      <c r="M39" s="15"/>
-      <c r="N39" s="15"/>
-      <c r="O39" s="16"/>
-      <c r="P39" s="16"/>
+      <c r="D39" s="18"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="18"/>
+      <c r="J39" s="18"/>
+      <c r="K39" s="18"/>
+      <c r="L39" s="18"/>
+      <c r="M39" s="18"/>
+      <c r="N39" s="18"/>
+      <c r="O39" s="19"/>
+      <c r="P39" s="19"/>
     </row>
     <row r="40" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C40" s="5"/>
-      <c r="D40" s="15"/>
-      <c r="E40" s="15"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15"/>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="15"/>
-      <c r="K40" s="15"/>
-      <c r="L40" s="15"/>
-      <c r="M40" s="15"/>
-      <c r="N40" s="15"/>
-      <c r="O40" s="16"/>
-      <c r="P40" s="16"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="18"/>
+      <c r="J40" s="18"/>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="18"/>
+      <c r="N40" s="18"/>
+      <c r="O40" s="19"/>
+      <c r="P40" s="19"/>
     </row>
     <row r="41" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C41" s="5"/>
-      <c r="D41" s="15"/>
-      <c r="E41" s="15"/>
-      <c r="F41" s="15"/>
-      <c r="G41" s="15"/>
-      <c r="H41" s="15"/>
-      <c r="I41" s="15"/>
-      <c r="J41" s="15"/>
-      <c r="K41" s="15"/>
-      <c r="L41" s="15"/>
-      <c r="M41" s="15"/>
-      <c r="N41" s="15"/>
-      <c r="O41" s="16"/>
-      <c r="P41" s="16"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="18"/>
+      <c r="J41" s="18"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
+      <c r="N41" s="18"/>
+      <c r="O41" s="19"/>
+      <c r="P41" s="19"/>
     </row>
     <row r="42" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C42" s="5"/>
-      <c r="D42" s="15"/>
-      <c r="E42" s="15"/>
-      <c r="F42" s="15"/>
-      <c r="G42" s="15"/>
-      <c r="H42" s="15"/>
-      <c r="I42" s="15"/>
-      <c r="J42" s="15"/>
-      <c r="K42" s="15"/>
-      <c r="L42" s="15"/>
-      <c r="M42" s="15"/>
-      <c r="N42" s="15"/>
-      <c r="O42" s="16"/>
-      <c r="P42" s="16"/>
+      <c r="D42" s="18"/>
+      <c r="E42" s="18"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="18"/>
+      <c r="J42" s="18"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="18"/>
+      <c r="M42" s="18"/>
+      <c r="N42" s="18"/>
+      <c r="O42" s="19"/>
+      <c r="P42" s="19"/>
     </row>
     <row r="43" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C43" s="5"/>
-      <c r="D43" s="15"/>
-      <c r="E43" s="15"/>
-      <c r="F43" s="15"/>
-      <c r="G43" s="15"/>
-      <c r="H43" s="15"/>
-      <c r="I43" s="15"/>
-      <c r="J43" s="15"/>
-      <c r="K43" s="15"/>
-      <c r="L43" s="15"/>
-      <c r="M43" s="15"/>
-      <c r="N43" s="15"/>
-      <c r="O43" s="16"/>
-      <c r="P43" s="16"/>
+      <c r="D43" s="18"/>
+      <c r="E43" s="18"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="18"/>
+      <c r="J43" s="18"/>
+      <c r="K43" s="18"/>
+      <c r="L43" s="18"/>
+      <c r="M43" s="18"/>
+      <c r="N43" s="18"/>
+      <c r="O43" s="19"/>
+      <c r="P43" s="19"/>
     </row>
     <row r="44" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C44" s="5"/>
-      <c r="D44" s="15"/>
-      <c r="E44" s="15"/>
-      <c r="F44" s="15"/>
-      <c r="G44" s="15"/>
-      <c r="H44" s="15"/>
-      <c r="I44" s="15"/>
-      <c r="J44" s="15"/>
-      <c r="K44" s="15"/>
-      <c r="L44" s="15"/>
-      <c r="M44" s="15"/>
-      <c r="N44" s="15"/>
-      <c r="O44" s="16"/>
-      <c r="P44" s="16"/>
+      <c r="D44" s="18"/>
+      <c r="E44" s="18"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="18"/>
+      <c r="J44" s="18"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="18"/>
+      <c r="M44" s="18"/>
+      <c r="N44" s="18"/>
+      <c r="O44" s="19"/>
+      <c r="P44" s="19"/>
     </row>
     <row r="45" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C45" s="5"/>
-      <c r="D45" s="15"/>
-      <c r="E45" s="15"/>
-      <c r="F45" s="15"/>
-      <c r="G45" s="15"/>
-      <c r="H45" s="15"/>
-      <c r="I45" s="15"/>
-      <c r="J45" s="15"/>
-      <c r="K45" s="15"/>
-      <c r="L45" s="15"/>
-      <c r="M45" s="15"/>
-      <c r="N45" s="15"/>
-      <c r="O45" s="16"/>
-      <c r="P45" s="16"/>
+      <c r="D45" s="18"/>
+      <c r="E45" s="18"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="18"/>
+      <c r="J45" s="18"/>
+      <c r="K45" s="18"/>
+      <c r="L45" s="18"/>
+      <c r="M45" s="18"/>
+      <c r="N45" s="18"/>
+      <c r="O45" s="19"/>
+      <c r="P45" s="19"/>
     </row>
     <row r="46" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C46" s="5"/>
-      <c r="D46" s="15"/>
-      <c r="E46" s="15"/>
-      <c r="F46" s="15"/>
-      <c r="G46" s="15"/>
-      <c r="H46" s="15"/>
-      <c r="I46" s="15"/>
-      <c r="J46" s="15"/>
-      <c r="K46" s="15"/>
-      <c r="L46" s="15"/>
-      <c r="M46" s="15"/>
-      <c r="N46" s="15"/>
-      <c r="O46" s="16"/>
-      <c r="P46" s="16"/>
+      <c r="D46" s="18"/>
+      <c r="E46" s="18"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="18"/>
+      <c r="J46" s="18"/>
+      <c r="K46" s="18"/>
+      <c r="L46" s="18"/>
+      <c r="M46" s="18"/>
+      <c r="N46" s="18"/>
+      <c r="O46" s="19"/>
+      <c r="P46" s="19"/>
     </row>
     <row r="47" spans="3:16" x14ac:dyDescent="0.3">
       <c r="C47" s="5"/>
-      <c r="D47" s="15"/>
-      <c r="E47" s="15"/>
-      <c r="F47" s="15"/>
-      <c r="G47" s="15"/>
-      <c r="H47" s="15"/>
-      <c r="I47" s="15"/>
-      <c r="J47" s="15"/>
-      <c r="K47" s="15"/>
-      <c r="L47" s="15"/>
-      <c r="M47" s="15"/>
-      <c r="N47" s="15"/>
-      <c r="O47" s="16"/>
-      <c r="P47" s="16"/>
+      <c r="D47" s="18"/>
+      <c r="E47" s="18"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="18"/>
+      <c r="J47" s="18"/>
+      <c r="K47" s="18"/>
+      <c r="L47" s="18"/>
+      <c r="M47" s="18"/>
+      <c r="N47" s="18"/>
+      <c r="O47" s="19"/>
+      <c r="P47" s="19"/>
     </row>
   </sheetData>
   <mergeCells count="187">

</xml_diff>